<commit_message>
Rework ZSD_EPACK into Excel-upload report with one form per packing list
- Parser splits the upload into packing lists (several per file),
  keeps header, invoices and items per packing list; 20 unit tests
- Data retrieval follows the FS logic sheet row by row and reads all
  SAP tables once per run for all packing lists (no SELECT in loops)
- One Smart Form call per packing list; a failing packing list is
  logged and does not stop the others
- Uploaded data saved to the Z tables after output; new log table
  ZSD_EPACK_LOG with one row per packing list
- Separate upload transaction withdrawn; design, field mapping, open
  questions and test plan in docs/Packing_List_Report_Design.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0112PqhqihbYdjNWGe6hooZE
</commit_message>
<xml_diff>
--- a/templates/ZSD_EPACK_Upload_Template_v2.xlsx
+++ b/templates/ZSD_EPACK_Upload_Template_v2.xlsx
@@ -8188,7 +8188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -8197,7 +8197,7 @@
     <row r="1">
       <c r="A1" s="46" t="inlineStr">
         <is>
-          <t>Export Packing List upload (transaction ZSD_EPACK_UPL) - template rules</t>
+          <t>Export Packing List - upload file for transaction ZSD_EPACK (one form per packing list)</t>
         </is>
       </c>
     </row>
@@ -8207,7 +8207,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Only the FIRST sheet ('Format') is uploaded. Keep the heading row (row 1) and the column order A-AL.</t>
+          <t>1. Only the FIRST sheet ('Format') is read. Keep the heading row (row 1) and the column order A-AL.</t>
         </is>
       </c>
     </row>
@@ -8221,120 +8221,141 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Header columns L-AK may be filled in any row (normally row 2). The same value may repeat in later rows; a different value is an error.</t>
+          <t>3. SEVERAL PACKING LISTS PER FILE: enter the Packing list no (column M) in the first row of each packing list.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4. Column L - SAP Invoice Number: all tax invoices of this packing list. One per row and/or several in one cell separated by , ; &amp; / or blanks.</t>
+          <t xml:space="preserve">   Rows with column M empty belong to the packing list of the nearest row above. Each packing list gets its own form.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5. Mandatory: Sl.No., Part No., Quantity on every line; Packing list no, Packing list date and at least one invoice.</t>
+          <t>4. Header columns N-AK of a packing list may be filled in any of its rows (normally the first). A repeated value must be identical.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6. Merged cells are allowed for Article No., Articles, Gross Wt. and Net Wt. (one package containing several materials).</t>
+          <t>5. Column L - SAP Invoice Number: all tax invoices of the packing list; one per row and/or several in one cell separated by , ; &amp; / or blanks.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Excel keeps the value in the first cell only: an empty Articles cell belongs to the group above, empty Gross+Net Wt. cells belong to the weight group above.</t>
+          <t xml:space="preserve">   Repeated numbers are counted once. One invoice may not appear under two packing lists.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Gross and Net Wt. must always be entered together. Gross Wt. must be &gt;= Net Wt. (FS rule).</t>
+          <t>6. Mandatory: Sl.No., Part No., Quantity on every line; Packing list no, Packing list date and at least one invoice per packing list.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>7. Quantity should equal STD x Articles - a difference is reported as a warning.</t>
+          <t>7. Merged cells are allowed for Article No., Articles, Gross Wt. and Net Wt. (one package containing several materials).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>8. Column AL Package Type (NEW, optional): Loose Pipes / Boxes / Bundles ... Enter it on the first line of each run of lines; it is carried forward.</t>
+          <t xml:space="preserve">   Excel keeps the value in the first cell only: an empty Articles cell belongs to the group above, empty Gross+Net Wt. cells to the weight group above.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   With more than one package type the printout shows subtotals ('2342 &lt;=Loose Pipes') and the total text 'Total 2342 Loose Pipes + 1073 Boxes = 3415 Packages'.</t>
+          <t xml:space="preserve">   Gross and Net Wt. are entered together. Gross Wt. must be &gt;= Net Wt. (FS rule) - otherwise no form is printed for that packing list.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9. Multi-line cells (Alt+Enter) are printed line by line: Notify parties, Container No, No. of Packages, Description of goods, Declaration.</t>
+          <t>8. Quantity should equal STD x Articles - a difference is reported as a warning.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10. Notify parties must be filled from 1 upwards (no gaps). If any notify party is filled, the format 'with notify party' is printed.</t>
+          <t>9. Column AL Package Type (NEW, optional): Loose Pipes / Boxes / Bundles ... entered on the first line of each run; carried forward.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11. Product Description (G) and H.S Code (K) may be left empty - they are then taken from the material master (MAKT / MARC-STEUC).</t>
+          <t>10. Multi-line cells (Alt+Enter) are printed line by line: notify parties, Container No, No. of Packages, Description of goods, Declaration.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12. Exporter Ref (O) may be left empty - the IEC is then taken from the company address in SAP.</t>
+          <t>11. Notify parties must be filled from 1 upwards. If any notify party is filled, the format 'with notify party' is printed.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>13. Description of goods (AG): one line per HSN, containing the HSN code (e.g. 'PVC PIPES (LEAD FREE) - HS CODE : 3917 2390'). The line is also used as section heading in the item table.</t>
+          <t>12. Product Description (G) and H.S Code (K) may be left empty - they are then taken from the material master of the Part No.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14. Dates: DD.MM.YYYY or an Excel date. Numbers: plain Excel numbers; weights are rounded to 3 decimals.</t>
+          <t>13. Column O (Exporter Ref) is not used - the IEC is read from the company address in SAP (FS logic sheet).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>15. Run the upload in TEST mode first. 'Overwrite' replaces an existing packing list and increases its revision number.</t>
+          <t>14. Description of goods (AG) may be left empty - it is then built from the HSN codes of the billed materials (FS logic sheet).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>15. Dates: DD.MM.YYYY or an Excel date. Numbers: plain Excel numbers; weights are rounded to 3 decimals.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
+        <is>
+          <t>16. Use 'Validate only' first. After a successful output the data is saved to the Z tables and a log row is written per packing list;</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    a packing list uploaded again replaces the saved one and gets the next revision number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>See sheet 'Example_90000081' for a filled example (data of PackingList_90000081 Nabil Yemen_BySea - Rev.1.pdf).</t>
         </is>

</xml_diff>